<commit_message>
Legg til Mørk GK i slopetabellen
Ny bane med 4 utslagssteder (Gul, Blå, Rød, Brun) for begge kjønn.
data.json regenerert fra Slopetabell.xlsx med convert-xlsx-to-json.ps1.
</commit_message>
<xml_diff>
--- a/Slopetabell.xlsx
+++ b/Slopetabell.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stian.VOM\Claude CODE\HCP kalkulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DC0EDF2-1625-4E41-8F1E-D4A2A6EB918A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740930A6-3C8C-4ACD-8180-23FDAF42B675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28275" yWindow="0" windowWidth="23430" windowHeight="20985" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="16">
   <si>
     <t>Bane</t>
   </si>
@@ -72,6 +72,21 @@
   </si>
   <si>
     <t>Dame</t>
+  </si>
+  <si>
+    <t>Mørk GK</t>
+  </si>
+  <si>
+    <t>Gul</t>
+  </si>
+  <si>
+    <t>Blå</t>
+  </si>
+  <si>
+    <t>Rød</t>
+  </si>
+  <si>
+    <t>Brun</t>
   </si>
 </sst>
 </file>
@@ -443,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77ED275-6173-40DF-A39D-63CFB668B5A5}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -565,6 +580,142 @@
         <v>115</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>71.5</v>
+      </c>
+      <c r="E8">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>69.3</v>
+      </c>
+      <c r="E9">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>67.8</v>
+      </c>
+      <c r="E10">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11">
+        <v>64</v>
+      </c>
+      <c r="E11">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="E12">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="E13">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="E14">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15">
+        <v>65.2</v>
+      </c>
+      <c r="E15">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Legg til Tjøme GK i slopetabellen
Ny bane med 4 utslagssteder (55, 50, 44, 32) for begge kjønn.
data.json regenerert fra Slopetabell.xlsx med convert-xlsx-to-json.ps1.
</commit_message>
<xml_diff>
--- a/Slopetabell.xlsx
+++ b/Slopetabell.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stian.VOM\Claude CODE\HCP kalkulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740930A6-3C8C-4ACD-8180-23FDAF42B675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559B479C-A0FB-44A8-B38D-C67430307BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28275" yWindow="0" windowWidth="23430" windowHeight="20985" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="7770" windowHeight="11370" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="17">
   <si>
     <t>Bane</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Brun</t>
+  </si>
+  <si>
+    <t>Tjøme GK</t>
   </si>
 </sst>
 </file>
@@ -458,10 +461,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77ED275-6173-40DF-A39D-63CFB668B5A5}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -478,7 +481,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -495,7 +498,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -512,7 +515,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -529,7 +532,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -546,7 +549,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -563,7 +566,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -580,7 +583,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -597,7 +600,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -614,7 +617,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -631,7 +634,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -648,7 +651,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -665,7 +668,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -682,7 +685,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -699,7 +702,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -714,6 +717,142 @@
       </c>
       <c r="E15">
         <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16">
+        <v>55</v>
+      </c>
+      <c r="D16">
+        <v>69.5</v>
+      </c>
+      <c r="E16">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>50</v>
+      </c>
+      <c r="D17">
+        <v>66.8</v>
+      </c>
+      <c r="E17">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18">
+        <v>44</v>
+      </c>
+      <c r="D18">
+        <v>64.3</v>
+      </c>
+      <c r="E18">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19">
+        <v>32</v>
+      </c>
+      <c r="D19">
+        <v>60.8</v>
+      </c>
+      <c r="E19">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20">
+        <v>55</v>
+      </c>
+      <c r="D20">
+        <v>75.400000000000006</v>
+      </c>
+      <c r="E20">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>50</v>
+      </c>
+      <c r="D21">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="E21">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22">
+        <v>44</v>
+      </c>
+      <c r="D22">
+        <v>68.900000000000006</v>
+      </c>
+      <c r="E22">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23">
+        <v>32</v>
+      </c>
+      <c r="D23">
+        <v>61.6</v>
+      </c>
+      <c r="E23">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Legg til Hakadal GK i slopetabellen
Ny bane med 5 utslagssteder (61, 57, 51, 47, 28) for begge kjønn.
data.json regenerert fra Slopetabell.xlsx med convert-xlsx-to-json.ps1.
</commit_message>
<xml_diff>
--- a/Slopetabell.xlsx
+++ b/Slopetabell.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stian.VOM\Claude CODE\HCP kalkulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559B479C-A0FB-44A8-B38D-C67430307BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0EAF84-A4F8-4177-AE47-15A67B2AA043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="7770" windowHeight="11370" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="18">
   <si>
     <t>Bane</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Tjøme GK</t>
+  </si>
+  <si>
+    <t>Hakadal GK</t>
   </si>
 </sst>
 </file>
@@ -461,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77ED275-6173-40DF-A39D-63CFB668B5A5}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -855,6 +858,176 @@
         <v>115</v>
       </c>
     </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24">
+        <v>61</v>
+      </c>
+      <c r="D24">
+        <v>72.5</v>
+      </c>
+      <c r="E24">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25">
+        <v>57</v>
+      </c>
+      <c r="D25">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="E25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26">
+        <v>51</v>
+      </c>
+      <c r="D26">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="E26">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27">
+        <v>47</v>
+      </c>
+      <c r="D27">
+        <v>65.2</v>
+      </c>
+      <c r="E27">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28">
+        <v>28</v>
+      </c>
+      <c r="D28">
+        <v>55</v>
+      </c>
+      <c r="E28">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29">
+        <v>61</v>
+      </c>
+      <c r="D29">
+        <v>78.8</v>
+      </c>
+      <c r="E29">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30">
+        <v>57</v>
+      </c>
+      <c r="D30">
+        <v>76</v>
+      </c>
+      <c r="E30">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31">
+        <v>51</v>
+      </c>
+      <c r="D31">
+        <v>71.900000000000006</v>
+      </c>
+      <c r="E31">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32">
+        <v>47</v>
+      </c>
+      <c r="D32">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="E32">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33">
+        <v>28</v>
+      </c>
+      <c r="D33">
+        <v>59</v>
+      </c>
+      <c r="E33">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Legg til Dynekilen GK og Strømstad GK i slopetabellen
Dynekilen GK: 2 utslagssteder (Gul, Rød) for begge kjønn.
Strømstad GK: 4 utslagssteder (Gul, Rød, Blå, Hvit) for begge kjønn.
data.json regenerert fra Slopetabell.xlsx med convert-xlsx-to-json.ps1.
</commit_message>
<xml_diff>
--- a/Slopetabell.xlsx
+++ b/Slopetabell.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stian.VOM\Claude CODE\HCP kalkulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0EAF84-A4F8-4177-AE47-15A67B2AA043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A2F13F-9B82-4897-A711-76A7CE8EF307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
+    <workbookView xWindow="26955" yWindow="3405" windowWidth="28455" windowHeight="15345" xr2:uid="{E7A5055B-2126-44E2-818B-3044C29F5FFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="21">
   <si>
     <t>Bane</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>Hakadal GK</t>
+  </si>
+  <si>
+    <t>Dynekilen GK</t>
+  </si>
+  <si>
+    <t>Strømstad GK</t>
+  </si>
+  <si>
+    <t>Hvit</t>
   </si>
 </sst>
 </file>
@@ -464,10 +473,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A77ED275-6173-40DF-A39D-63CFB668B5A5}">
-  <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -484,7 +496,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -501,7 +513,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -518,7 +530,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -535,7 +547,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -552,7 +564,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -569,7 +581,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -586,7 +598,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -603,7 +615,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -620,7 +632,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -637,7 +649,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -654,7 +666,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -671,7 +683,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -688,7 +700,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -705,7 +717,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -722,7 +734,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -739,7 +751,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -756,7 +768,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -773,7 +785,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -790,7 +802,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -807,7 +819,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -824,7 +836,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -841,7 +853,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -858,7 +870,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -875,7 +887,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -892,7 +904,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -909,7 +921,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -926,7 +938,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -943,7 +955,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -960,7 +972,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>10</v>
       </c>
@@ -977,7 +989,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -994,7 +1006,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1011,7 +1023,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -1026,6 +1038,210 @@
       </c>
       <c r="E33">
         <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34">
+        <v>69.7</v>
+      </c>
+      <c r="E34">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35">
+        <v>65.2</v>
+      </c>
+      <c r="E35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36">
+        <v>75.400000000000006</v>
+      </c>
+      <c r="E36">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="E37">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38">
+        <v>69</v>
+      </c>
+      <c r="E38">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="E39">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>9</v>
+      </c>
+      <c r="B40" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40">
+        <v>67.2</v>
+      </c>
+      <c r="E40">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B41" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41">
+        <v>70.2</v>
+      </c>
+      <c r="E41">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42">
+        <v>74.8</v>
+      </c>
+      <c r="E42">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43">
+        <v>69.8</v>
+      </c>
+      <c r="E43">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>10</v>
+      </c>
+      <c r="B44" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44">
+        <v>65.599999999999994</v>
+      </c>
+      <c r="E44">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45">
+        <v>72</v>
+      </c>
+      <c r="E45">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>